<commit_message>
Formularer til person og virksomhed med dubletadvarsel, mellemnavn, sortering på for- og efternavn
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JipmKYTwY2CKcxt3AmMJgx
</commit_message>
<xml_diff>
--- a/docs/import_skabelon.xlsx
+++ b/docs/import_skabelon.xlsx
@@ -525,7 +525,6 @@
           <t>Entreprenør / Totalentreprenør</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>https://eksempel.example</t>
@@ -541,7 +540,6 @@
           <t>8000</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>TEST Eksempel Koncern</t>
@@ -552,7 +550,6 @@
           <t>Moderselskab</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -565,11 +562,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -594,75 +591,80 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Mellemnavn</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Efternavn</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>E-mail</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Telefon</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Virksomhed</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Tilknytning</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Niveau</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Funktion</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Slut</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Primær</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Kendskab</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Kendt siden</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Ingen invitation</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Noter</t>
         </is>
@@ -674,57 +676,53 @@
           <t>TEST Eksempel</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>eksempel@test.example</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>TEST Eksempel A/S</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Ansættelse</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Chef</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Ledelse</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Kender godt</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>2022-05-01</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Privat note</t>
         </is>

</xml_diff>